<commit_message>
Actualizar mapeo regional a COSTA, SIERRA y AMAZONIA
</commit_message>
<xml_diff>
--- a/INVENTARIOS AUTODECER.xlsx
+++ b/INVENTARIOS AUTODECER.xlsx
@@ -2707,10 +2707,8 @@
         </is>
       </c>
       <c r="B12" s="43" t="n"/>
-      <c r="C12" s="43" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C12" s="43" t="n">
+        <v>2</v>
       </c>
       <c r="D12" s="146" t="n"/>
       <c r="E12" s="133" t="n"/>

</xml_diff>